<commit_message>
aggiunto prototipo mostra cartucce
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\giuseppe\Desktop\Buckshot-Ruolette\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7496B9C0-F7F2-4BF6-A027-1CA2591B2E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E07EE04-8EF6-4E8A-83D3-94CE83493628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CBC2A017-6F82-4655-8A6A-84493A23D819}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>QUANTITà</t>
   </si>
@@ -84,6 +84,21 @@
   </si>
   <si>
     <t>speaker</t>
+  </si>
+  <si>
+    <t>inserti filettati per stampe3D M3</t>
+  </si>
+  <si>
+    <t>alimentatore 24v</t>
+  </si>
+  <si>
+    <t>alimentatore 5v</t>
+  </si>
+  <si>
+    <t>Unità TENS</t>
+  </si>
+  <si>
+    <t>scheda relè</t>
   </si>
 </sst>
 </file>
@@ -620,43 +635,58 @@
       <c r="A15" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="C16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="C17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="C18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="b">
         <v>0</v>
       </c>

</xml_diff>